<commit_message>
Modificacion del dataset a datos maximos diarios. Reentreno del modelo
</commit_message>
<xml_diff>
--- a/datos_lluvia_aemet/Arroyo.xlsx
+++ b/datos_lluvia_aemet/Arroyo.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B2224"/>
+  <dimension ref="A1:B2309"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -22610,6 +22610,848 @@
         <v>0.6</v>
       </c>
     </row>
+    <row r="2225">
+      <c r="A2225" t="inlineStr">
+        <is>
+          <t>01/02/2026</t>
+        </is>
+      </c>
+      <c r="B2225" t="n">
+        <v>4.6</v>
+      </c>
+    </row>
+    <row r="2226">
+      <c r="A2226" t="inlineStr">
+        <is>
+          <t>02/02/2026</t>
+        </is>
+      </c>
+      <c r="B2226" t="n">
+        <v>4.2</v>
+      </c>
+    </row>
+    <row r="2227">
+      <c r="A2227" t="inlineStr">
+        <is>
+          <t>03/02/2026</t>
+        </is>
+      </c>
+      <c r="B2227" t="n">
+        <v>1.8</v>
+      </c>
+    </row>
+    <row r="2228">
+      <c r="A2228" t="inlineStr">
+        <is>
+          <t>04/02/2026</t>
+        </is>
+      </c>
+      <c r="B2228" t="n">
+        <v>1.8</v>
+      </c>
+    </row>
+    <row r="2229">
+      <c r="A2229" t="inlineStr">
+        <is>
+          <t>05/02/2026</t>
+        </is>
+      </c>
+      <c r="B2229" t="n">
+        <v>5.8</v>
+      </c>
+    </row>
+    <row r="2230">
+      <c r="A2230" t="inlineStr">
+        <is>
+          <t>06/02/2026</t>
+        </is>
+      </c>
+      <c r="B2230" t="n">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="2231">
+      <c r="A2231" t="inlineStr">
+        <is>
+          <t>07/02/2026</t>
+        </is>
+      </c>
+      <c r="B2231" t="n">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="2232">
+      <c r="A2232" t="inlineStr">
+        <is>
+          <t>08/02/2026</t>
+        </is>
+      </c>
+      <c r="B2232" t="n">
+        <v>6.6</v>
+      </c>
+    </row>
+    <row r="2233">
+      <c r="A2233" t="inlineStr">
+        <is>
+          <t>09/02/2026</t>
+        </is>
+      </c>
+      <c r="B2233" t="n">
+        <v>3.8</v>
+      </c>
+    </row>
+    <row r="2234">
+      <c r="A2234" t="inlineStr">
+        <is>
+          <t>10/02/2026</t>
+        </is>
+      </c>
+      <c r="B2234" t="n">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="2235">
+      <c r="A2235" t="inlineStr">
+        <is>
+          <t>11/02/2026</t>
+        </is>
+      </c>
+      <c r="B2235" t="n">
+        <v>9.199999999999999</v>
+      </c>
+    </row>
+    <row r="2236">
+      <c r="A2236" t="inlineStr">
+        <is>
+          <t>12/02/2026</t>
+        </is>
+      </c>
+      <c r="B2236" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2237">
+      <c r="A2237" t="inlineStr">
+        <is>
+          <t>13/02/2026</t>
+        </is>
+      </c>
+      <c r="B2237" t="n">
+        <v>24.4</v>
+      </c>
+    </row>
+    <row r="2238">
+      <c r="A2238" t="inlineStr">
+        <is>
+          <t>14/02/2026</t>
+        </is>
+      </c>
+      <c r="B2238" t="n">
+        <v>8.4</v>
+      </c>
+    </row>
+    <row r="2239">
+      <c r="A2239" t="inlineStr">
+        <is>
+          <t>15/02/2026</t>
+        </is>
+      </c>
+      <c r="B2239" t="n">
+        <v>1.4</v>
+      </c>
+    </row>
+    <row r="2240">
+      <c r="A2240" t="inlineStr">
+        <is>
+          <t>16/02/2026</t>
+        </is>
+      </c>
+      <c r="B2240" t="n">
+        <v>16.2</v>
+      </c>
+    </row>
+    <row r="2241">
+      <c r="A2241" t="inlineStr">
+        <is>
+          <t>17/02/2026</t>
+        </is>
+      </c>
+      <c r="B2241" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2242">
+      <c r="A2242" t="inlineStr">
+        <is>
+          <t>18/02/2026</t>
+        </is>
+      </c>
+      <c r="B2242" t="n">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="2243">
+      <c r="A2243" t="inlineStr">
+        <is>
+          <t>19/02/2026</t>
+        </is>
+      </c>
+      <c r="B2243" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2244">
+      <c r="A2244" t="inlineStr">
+        <is>
+          <t>20/02/2026</t>
+        </is>
+      </c>
+      <c r="B2244" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2245">
+      <c r="A2245" t="inlineStr">
+        <is>
+          <t>21/02/2026</t>
+        </is>
+      </c>
+      <c r="B2245" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2246">
+      <c r="A2246" t="inlineStr">
+        <is>
+          <t>22/02/2026</t>
+        </is>
+      </c>
+      <c r="B2246" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2247">
+      <c r="A2247" t="inlineStr">
+        <is>
+          <t>23/02/2026</t>
+        </is>
+      </c>
+      <c r="B2247" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2248">
+      <c r="A2248" t="inlineStr">
+        <is>
+          <t>24/02/2026</t>
+        </is>
+      </c>
+      <c r="B2248" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2249">
+      <c r="A2249" t="inlineStr">
+        <is>
+          <t>25/02/2026</t>
+        </is>
+      </c>
+      <c r="B2249" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2250">
+      <c r="A2250" t="inlineStr">
+        <is>
+          <t>26/02/2026</t>
+        </is>
+      </c>
+      <c r="B2250" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2251">
+      <c r="A2251" t="inlineStr">
+        <is>
+          <t>27/02/2026</t>
+        </is>
+      </c>
+      <c r="B2251" t="n">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="2252">
+      <c r="A2252" t="inlineStr">
+        <is>
+          <t>28/02/2026</t>
+        </is>
+      </c>
+      <c r="B2252" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2253">
+      <c r="A2253" t="inlineStr">
+        <is>
+          <t>01/03/2026</t>
+        </is>
+      </c>
+      <c r="B2253" t="n">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="2254">
+      <c r="A2254" t="inlineStr">
+        <is>
+          <t>02/03/2026</t>
+        </is>
+      </c>
+      <c r="B2254" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2255">
+      <c r="A2255" t="inlineStr">
+        <is>
+          <t>03/03/2026</t>
+        </is>
+      </c>
+      <c r="B2255" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2256">
+      <c r="A2256" t="inlineStr">
+        <is>
+          <t>04/03/2026</t>
+        </is>
+      </c>
+      <c r="B2256" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2257">
+      <c r="A2257" t="inlineStr">
+        <is>
+          <t>05/03/2026</t>
+        </is>
+      </c>
+      <c r="B2257" t="n">
+        <v>3.4</v>
+      </c>
+    </row>
+    <row r="2258">
+      <c r="A2258" t="inlineStr">
+        <is>
+          <t>06/03/2026</t>
+        </is>
+      </c>
+      <c r="B2258" t="n">
+        <v>2.8</v>
+      </c>
+    </row>
+    <row r="2259">
+      <c r="A2259" t="inlineStr">
+        <is>
+          <t>07/03/2026</t>
+        </is>
+      </c>
+      <c r="B2259" t="n">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="2260">
+      <c r="A2260" t="inlineStr">
+        <is>
+          <t>08/03/2026</t>
+        </is>
+      </c>
+      <c r="B2260" t="n">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="2261">
+      <c r="A2261" t="inlineStr">
+        <is>
+          <t>09/03/2026</t>
+        </is>
+      </c>
+      <c r="B2261" t="n">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="2262">
+      <c r="A2262" t="inlineStr">
+        <is>
+          <t>10/03/2026</t>
+        </is>
+      </c>
+      <c r="B2262" t="n">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="2263">
+      <c r="A2263" t="inlineStr">
+        <is>
+          <t>11/03/2026</t>
+        </is>
+      </c>
+      <c r="B2263" t="inlineStr"/>
+    </row>
+    <row r="2264">
+      <c r="A2264" t="inlineStr">
+        <is>
+          <t>12/03/2026</t>
+        </is>
+      </c>
+      <c r="B2264" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2265">
+      <c r="A2265" t="inlineStr">
+        <is>
+          <t>13/03/2026</t>
+        </is>
+      </c>
+      <c r="B2265" t="n">
+        <v>5.4</v>
+      </c>
+    </row>
+    <row r="2266">
+      <c r="A2266" t="inlineStr">
+        <is>
+          <t>14/03/2026</t>
+        </is>
+      </c>
+      <c r="B2266" t="n">
+        <v>16.4</v>
+      </c>
+    </row>
+    <row r="2267">
+      <c r="A2267" t="inlineStr">
+        <is>
+          <t>15/03/2026</t>
+        </is>
+      </c>
+      <c r="B2267" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2268">
+      <c r="A2268" t="inlineStr">
+        <is>
+          <t>16/03/2026</t>
+        </is>
+      </c>
+      <c r="B2268" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2269">
+      <c r="A2269" t="inlineStr">
+        <is>
+          <t>17/03/2026</t>
+        </is>
+      </c>
+      <c r="B2269" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2270">
+      <c r="A2270" t="inlineStr">
+        <is>
+          <t>18/03/2026</t>
+        </is>
+      </c>
+      <c r="B2270" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2271">
+      <c r="A2271" t="inlineStr">
+        <is>
+          <t>19/03/2026</t>
+        </is>
+      </c>
+      <c r="B2271" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2272">
+      <c r="A2272" t="inlineStr">
+        <is>
+          <t>20/03/2026</t>
+        </is>
+      </c>
+      <c r="B2272" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2273">
+      <c r="A2273" t="inlineStr">
+        <is>
+          <t>21/03/2026</t>
+        </is>
+      </c>
+      <c r="B2273" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2274">
+      <c r="A2274" t="inlineStr">
+        <is>
+          <t>22/03/2026</t>
+        </is>
+      </c>
+      <c r="B2274" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2275">
+      <c r="A2275" t="inlineStr">
+        <is>
+          <t>23/03/2026</t>
+        </is>
+      </c>
+      <c r="B2275" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2276">
+      <c r="A2276" t="inlineStr">
+        <is>
+          <t>24/03/2026</t>
+        </is>
+      </c>
+      <c r="B2276" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2277">
+      <c r="A2277" t="inlineStr">
+        <is>
+          <t>25/03/2026</t>
+        </is>
+      </c>
+      <c r="B2277" t="n">
+        <v>4.4</v>
+      </c>
+    </row>
+    <row r="2278">
+      <c r="A2278" t="inlineStr">
+        <is>
+          <t>26/03/2026</t>
+        </is>
+      </c>
+      <c r="B2278" t="n">
+        <v>4.4</v>
+      </c>
+    </row>
+    <row r="2279">
+      <c r="A2279" t="inlineStr">
+        <is>
+          <t>27/03/2026</t>
+        </is>
+      </c>
+      <c r="B2279" t="n">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="2280">
+      <c r="A2280" t="inlineStr">
+        <is>
+          <t>28/03/2026</t>
+        </is>
+      </c>
+      <c r="B2280" t="n">
+        <v>5.6</v>
+      </c>
+    </row>
+    <row r="2281">
+      <c r="A2281" t="inlineStr">
+        <is>
+          <t>29/03/2026</t>
+        </is>
+      </c>
+      <c r="B2281" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2282">
+      <c r="A2282" t="inlineStr">
+        <is>
+          <t>30/03/2026</t>
+        </is>
+      </c>
+      <c r="B2282" t="n">
+        <v>5.8</v>
+      </c>
+    </row>
+    <row r="2283">
+      <c r="A2283" t="inlineStr">
+        <is>
+          <t>31/03/2026</t>
+        </is>
+      </c>
+      <c r="B2283" t="n">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="2284">
+      <c r="A2284" t="inlineStr">
+        <is>
+          <t>01/04/2026</t>
+        </is>
+      </c>
+      <c r="B2284" t="n">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="2285">
+      <c r="A2285" t="inlineStr">
+        <is>
+          <t>02/04/2026</t>
+        </is>
+      </c>
+      <c r="B2285" t="n">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="2286">
+      <c r="A2286" t="inlineStr">
+        <is>
+          <t>03/04/2026</t>
+        </is>
+      </c>
+      <c r="B2286" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2287">
+      <c r="A2287" t="inlineStr">
+        <is>
+          <t>04/04/2026</t>
+        </is>
+      </c>
+      <c r="B2287" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2288">
+      <c r="A2288" t="inlineStr">
+        <is>
+          <t>05/04/2026</t>
+        </is>
+      </c>
+      <c r="B2288" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2289">
+      <c r="A2289" t="inlineStr">
+        <is>
+          <t>06/04/2026</t>
+        </is>
+      </c>
+      <c r="B2289" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2290">
+      <c r="A2290" t="inlineStr">
+        <is>
+          <t>07/04/2026</t>
+        </is>
+      </c>
+      <c r="B2290" t="n">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="2291">
+      <c r="A2291" t="inlineStr">
+        <is>
+          <t>08/04/2026</t>
+        </is>
+      </c>
+      <c r="B2291" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2292">
+      <c r="A2292" t="inlineStr">
+        <is>
+          <t>09/04/2026</t>
+        </is>
+      </c>
+      <c r="B2292" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2293">
+      <c r="A2293" t="inlineStr">
+        <is>
+          <t>10/04/2026</t>
+        </is>
+      </c>
+      <c r="B2293" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2294">
+      <c r="A2294" t="inlineStr">
+        <is>
+          <t>11/04/2026</t>
+        </is>
+      </c>
+      <c r="B2294" t="n">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="2295">
+      <c r="A2295" t="inlineStr">
+        <is>
+          <t>12/04/2026</t>
+        </is>
+      </c>
+      <c r="B2295" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2296">
+      <c r="A2296" t="inlineStr">
+        <is>
+          <t>13/04/2026</t>
+        </is>
+      </c>
+      <c r="B2296" t="n">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="2297">
+      <c r="A2297" t="inlineStr">
+        <is>
+          <t>14/04/2026</t>
+        </is>
+      </c>
+      <c r="B2297" t="n">
+        <v>1.8</v>
+      </c>
+    </row>
+    <row r="2298">
+      <c r="A2298" t="inlineStr">
+        <is>
+          <t>15/04/2026</t>
+        </is>
+      </c>
+      <c r="B2298" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2299">
+      <c r="A2299" t="inlineStr">
+        <is>
+          <t>16/04/2026</t>
+        </is>
+      </c>
+      <c r="B2299" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2300">
+      <c r="A2300" t="inlineStr">
+        <is>
+          <t>17/04/2026</t>
+        </is>
+      </c>
+      <c r="B2300" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2301">
+      <c r="A2301" t="inlineStr">
+        <is>
+          <t>18/04/2026</t>
+        </is>
+      </c>
+      <c r="B2301" t="n">
+        <v>8.800000000000001</v>
+      </c>
+    </row>
+    <row r="2302">
+      <c r="A2302" t="inlineStr">
+        <is>
+          <t>19/04/2026</t>
+        </is>
+      </c>
+      <c r="B2302" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2303">
+      <c r="A2303" t="inlineStr">
+        <is>
+          <t>20/04/2026</t>
+        </is>
+      </c>
+      <c r="B2303" t="n">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="2304">
+      <c r="A2304" t="inlineStr">
+        <is>
+          <t>21/04/2026</t>
+        </is>
+      </c>
+      <c r="B2304" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2305">
+      <c r="A2305" t="inlineStr">
+        <is>
+          <t>22/04/2026</t>
+        </is>
+      </c>
+      <c r="B2305" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2306">
+      <c r="A2306" t="inlineStr">
+        <is>
+          <t>23/04/2026</t>
+        </is>
+      </c>
+      <c r="B2306" t="n">
+        <v>2.8</v>
+      </c>
+    </row>
+    <row r="2307">
+      <c r="A2307" t="inlineStr">
+        <is>
+          <t>24/04/2026</t>
+        </is>
+      </c>
+      <c r="B2307" t="inlineStr"/>
+    </row>
+    <row r="2308">
+      <c r="A2308" t="inlineStr">
+        <is>
+          <t>25/04/2026</t>
+        </is>
+      </c>
+      <c r="B2308" t="inlineStr"/>
+    </row>
+    <row r="2309">
+      <c r="A2309" t="inlineStr">
+        <is>
+          <t>26/04/2026</t>
+        </is>
+      </c>
+      <c r="B2309" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>